<commit_message>
feat(certificates): clean demo records, enable Cloudinary template upload, replacement, and deletion
</commit_message>
<xml_diff>
--- a/data/attendees.xlsx
+++ b/data/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,109 +419,9 @@
         <v>Certificate ID</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>0108CS221001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Aarav Sharma</v>
-      </c>
-      <c r="C2" t="str">
-        <v>National Cyber Defense Wargame 2026</v>
-      </c>
-      <c r="D2" t="str">
-        <v>1st Place Winner</v>
-      </c>
-      <c r="E2" t="str">
-        <v>2026-10-19</v>
-      </c>
-      <c r="F2" t="str">
-        <v>CYB-2026-ARV001</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>0108CS221045</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Yash Harfode</v>
-      </c>
-      <c r="C3" t="str">
-        <v>National Cyber Defense Wargame 2026</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Lead Convenor</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-10-19</v>
-      </c>
-      <c r="F3" t="str">
-        <v>CYB-2026-YSH045</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>0108IT221012</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Priya Sen</v>
-      </c>
-      <c r="C4" t="str">
-        <v>National Cyber Defense Wargame 2026</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2nd Place Winner</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2026-10-19</v>
-      </c>
-      <c r="F4" t="str">
-        <v>CYB-2026-PRY012</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>0108EC221089</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Rohan Vishwakarma</v>
-      </c>
-      <c r="C5" t="str">
-        <v>National Cyber Defense Wargame 2026</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Participant</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-10-19</v>
-      </c>
-      <c r="F5" t="str">
-        <v>CYB-2026-RHN089</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>0108CS221099</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Ananya Joshi</v>
-      </c>
-      <c r="C6" t="str">
-        <v>National Cyber Defense Wargame 2026</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Participant</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-10-19</v>
-      </c>
-      <c r="F6" t="str">
-        <v>CYB-2026-ANA099</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>